<commit_message>
Aggiornato Avanzamento.xlsx da lbianco via Streamlit
</commit_message>
<xml_diff>
--- a/Avanzamento.xlsx
+++ b/Avanzamento.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="154">
   <si>
     <t>Tecnico</t>
   </si>
@@ -599,14 +599,12 @@
       <alignment horizontal="right" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -902,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H345"/>
+  <dimension ref="A1:H343"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
@@ -7636,7 +7634,7 @@
         <v>20</v>
       </c>
       <c r="F272" s="3">
-        <f t="shared" ref="F272:F338" si="6">D272-(D272*E272)/100</f>
+        <f t="shared" ref="F272:F336" si="6">D272-(D272*E272)/100</f>
         <v>36.681839742579442</v>
       </c>
       <c r="G272" s="1"/>
@@ -7647,22 +7645,22 @@
         <v>4</v>
       </c>
       <c r="B273" s="11">
-        <v>45979</v>
-      </c>
-      <c r="C273" s="12">
-        <v>60</v>
-      </c>
-      <c r="D273" s="13">
-        <v>29.346096938775499</v>
-      </c>
-      <c r="E273" s="14">
-        <v>20</v>
-      </c>
-      <c r="F273" s="15">
+        <v>45991</v>
+      </c>
+      <c r="C273" s="9">
+        <v>124</v>
+      </c>
+      <c r="D273" s="12">
+        <v>31.189142473118299</v>
+      </c>
+      <c r="E273" s="13">
+        <v>20</v>
+      </c>
+      <c r="F273" s="14">
         <f t="shared" si="6"/>
-        <v>23.476877551020401</v>
-      </c>
-      <c r="G273" s="10" t="s">
+        <v>24.951313978494639</v>
+      </c>
+      <c r="G273" s="15" t="s">
         <v>67</v>
       </c>
       <c r="H273" s="16" t="s">
@@ -7674,20 +7672,20 @@
         <v>5</v>
       </c>
       <c r="B274" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C274" s="9">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="D274" s="4">
-        <v>28.6650595515537</v>
+        <v>37.811625817847897</v>
       </c>
       <c r="E274" s="6">
         <v>20</v>
       </c>
       <c r="F274" s="3">
         <f t="shared" si="6"/>
-        <v>22.93204764124296</v>
+        <v>30.249300654278318</v>
       </c>
       <c r="G274" s="1" t="s">
         <v>67</v>
@@ -7701,16 +7699,20 @@
         <v>139</v>
       </c>
       <c r="B275" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C275" s="9"/>
-      <c r="D275" s="4"/>
+        <v>45991</v>
+      </c>
+      <c r="C275" s="9">
+        <v>48</v>
+      </c>
+      <c r="D275" s="4">
+        <v>134.20636002328999</v>
+      </c>
       <c r="E275" s="6">
         <v>20</v>
       </c>
       <c r="F275" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>107.36508801863199</v>
       </c>
       <c r="G275" s="1"/>
       <c r="H275" s="8"/>
@@ -7720,20 +7722,20 @@
         <v>6</v>
       </c>
       <c r="B276" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C276" s="9">
-        <v>69</v>
+        <v>141</v>
       </c>
       <c r="D276" s="4">
-        <v>43.425407592332903</v>
+        <v>31.485793439459201</v>
       </c>
       <c r="E276" s="6">
         <v>20</v>
       </c>
       <c r="F276" s="3">
         <f t="shared" si="6"/>
-        <v>34.740326073866321</v>
+        <v>25.18863475156736</v>
       </c>
       <c r="G276" s="1"/>
       <c r="H276" s="8" t="s">
@@ -7745,20 +7747,20 @@
         <v>7</v>
       </c>
       <c r="B277" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C277" s="9">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D277" s="4">
-        <v>791.60524999999996</v>
+        <v>203.80709722222201</v>
       </c>
       <c r="E277" s="6">
         <v>20</v>
       </c>
       <c r="F277" s="3">
         <f t="shared" si="6"/>
-        <v>633.28419999999994</v>
+        <v>163.0456777777776</v>
       </c>
       <c r="G277" s="1"/>
       <c r="H277" s="8" t="s">
@@ -7770,20 +7772,20 @@
         <v>8</v>
       </c>
       <c r="B278" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C278" s="9">
-        <v>88</v>
+        <v>152</v>
       </c>
       <c r="D278" s="4">
-        <v>27.603030921459499</v>
+        <v>29.248444138400199</v>
       </c>
       <c r="E278" s="6">
         <v>20</v>
       </c>
       <c r="F278" s="3">
         <f t="shared" si="6"/>
-        <v>22.082424737167599</v>
+        <v>23.398755310720158</v>
       </c>
       <c r="G278" s="1"/>
       <c r="H278" s="8" t="s">
@@ -7795,20 +7797,20 @@
         <v>9</v>
       </c>
       <c r="B279" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C279" s="9">
-        <v>87</v>
+        <v>135</v>
       </c>
       <c r="D279" s="4">
-        <v>32.3825986394558</v>
+        <v>39.744967680608397</v>
       </c>
       <c r="E279" s="6">
         <v>20</v>
       </c>
       <c r="F279" s="3">
         <f t="shared" si="6"/>
-        <v>25.906078911564641</v>
+        <v>31.795974144486717</v>
       </c>
       <c r="G279" s="1"/>
       <c r="H279" s="8" t="s">
@@ -7820,20 +7822,20 @@
         <v>10</v>
       </c>
       <c r="B280" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C280" s="9">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="D280" s="4">
-        <v>34.770215</v>
+        <v>35.579655487804899</v>
       </c>
       <c r="E280" s="6">
         <v>20</v>
       </c>
       <c r="F280" s="3">
         <f t="shared" si="6"/>
-        <v>27.816172000000002</v>
+        <v>28.463724390243918</v>
       </c>
       <c r="G280" s="1"/>
       <c r="H280" s="8" t="s">
@@ -7845,20 +7847,20 @@
         <v>11</v>
       </c>
       <c r="B281" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C281" s="9">
-        <v>95</v>
+        <v>159</v>
       </c>
       <c r="D281" s="4">
-        <v>32.3825986394558</v>
+        <v>39.744967680608397</v>
       </c>
       <c r="E281" s="6">
         <v>20</v>
       </c>
       <c r="F281" s="3">
         <f t="shared" si="6"/>
-        <v>25.906078911564641</v>
+        <v>31.795974144486717</v>
       </c>
       <c r="G281" s="1"/>
       <c r="H281" s="8" t="s">
@@ -7870,20 +7872,20 @@
         <v>12</v>
       </c>
       <c r="B282" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C282" s="9">
-        <v>110</v>
+        <v>182</v>
       </c>
       <c r="D282" s="4">
-        <v>24.5925847457627</v>
+        <v>56.329923570077497</v>
       </c>
       <c r="E282" s="6">
         <v>20</v>
       </c>
       <c r="F282" s="3">
         <f t="shared" si="6"/>
-        <v>19.67406779661016</v>
+        <v>45.063938856061995</v>
       </c>
       <c r="G282" s="1"/>
       <c r="H282" s="8" t="s">
@@ -7895,20 +7897,20 @@
         <v>13</v>
       </c>
       <c r="B283" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C283" s="9">
-        <v>110</v>
+        <v>182</v>
       </c>
       <c r="D283" s="4">
-        <v>24.5925847457627</v>
+        <v>56.329923570077497</v>
       </c>
       <c r="E283" s="6">
         <v>20</v>
       </c>
       <c r="F283" s="3">
         <f t="shared" si="6"/>
-        <v>19.67406779661016</v>
+        <v>45.063938856061995</v>
       </c>
       <c r="G283" s="1"/>
       <c r="H283" s="8" t="s">
@@ -7920,20 +7922,20 @@
         <v>14</v>
       </c>
       <c r="B284" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C284" s="9">
-        <v>88</v>
+        <v>160</v>
       </c>
       <c r="D284" s="4">
-        <v>52.361870530303001</v>
+        <v>42.655002724037701</v>
       </c>
       <c r="E284" s="6">
         <v>20</v>
       </c>
       <c r="F284" s="3">
         <f t="shared" si="6"/>
-        <v>41.889496424242402</v>
+        <v>34.12400217923016</v>
       </c>
       <c r="G284" s="1"/>
       <c r="H284" s="8" t="s">
@@ -7942,1490 +7944,1456 @@
     </row>
     <row r="285" spans="1:8">
       <c r="A285" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B285" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C285" s="9"/>
-      <c r="D285" s="4"/>
+        <v>45991</v>
+      </c>
+      <c r="C285" s="9">
+        <v>168</v>
+      </c>
+      <c r="D285" s="4">
+        <v>30.141696688279701</v>
+      </c>
       <c r="E285" s="6">
         <v>20</v>
       </c>
       <c r="F285" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>24.113357350623762</v>
       </c>
       <c r="G285" s="1"/>
       <c r="H285" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="286" spans="1:8">
       <c r="A286" s="1" t="s">
-        <v>16</v>
+        <v>151</v>
       </c>
       <c r="B286" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C286" s="9">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="D286" s="4">
-        <v>27.748286422902499</v>
+        <v>118.816192483051</v>
       </c>
       <c r="E286" s="6">
         <v>20</v>
       </c>
       <c r="F286" s="3">
         <f t="shared" si="6"/>
-        <v>22.198629138321998</v>
+        <v>95.052953986440798</v>
       </c>
       <c r="G286" s="1"/>
-      <c r="H286" s="8" t="s">
-        <v>87</v>
-      </c>
+      <c r="H286" s="8"/>
     </row>
     <row r="287" spans="1:8">
       <c r="A287" s="1" t="s">
-        <v>151</v>
+        <v>17</v>
       </c>
       <c r="B287" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C287" s="9">
-        <v>61</v>
+        <v>136</v>
       </c>
       <c r="D287" s="4">
-        <v>98.040274962742203</v>
+        <v>37.687197916666697</v>
       </c>
       <c r="E287" s="6">
         <v>20</v>
       </c>
       <c r="F287" s="3">
         <f t="shared" si="6"/>
-        <v>78.432219970193756</v>
+        <v>30.149758333333359</v>
       </c>
       <c r="G287" s="1"/>
-      <c r="H287" s="8"/>
+      <c r="H287" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="288" spans="1:8">
       <c r="A288" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B288" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C288" s="9">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="D288" s="4">
-        <v>35.915104166666701</v>
+        <v>34.291203234185197</v>
       </c>
       <c r="E288" s="6">
         <v>20</v>
       </c>
       <c r="F288" s="3">
         <f t="shared" si="6"/>
-        <v>28.73208333333336</v>
+        <v>27.432962587348158</v>
       </c>
       <c r="G288" s="1"/>
       <c r="H288" s="8" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="289" spans="1:8">
       <c r="A289" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B289" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C289" s="9">
-        <v>88</v>
+        <v>172</v>
       </c>
       <c r="D289" s="4">
-        <v>28.036716018884501</v>
+        <v>33.499415518672699</v>
       </c>
       <c r="E289" s="6">
         <v>20</v>
       </c>
       <c r="F289" s="3">
         <f t="shared" si="6"/>
-        <v>22.429372815107602</v>
+        <v>26.79953241493816</v>
       </c>
       <c r="G289" s="1"/>
       <c r="H289" s="8" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
     </row>
     <row r="290" spans="1:8">
       <c r="A290" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B290" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C290" s="9"/>
-      <c r="D290" s="4"/>
+        <v>45991</v>
+      </c>
+      <c r="C290" s="9">
+        <v>176</v>
+      </c>
+      <c r="D290" s="4">
+        <v>34.022932412626503</v>
+      </c>
       <c r="E290" s="6">
         <v>20</v>
       </c>
       <c r="F290" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>27.218345930101201</v>
       </c>
       <c r="G290" s="1"/>
       <c r="H290" s="8" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="291" spans="1:8">
-      <c r="A291" s="1" t="s">
-        <v>20</v>
+      <c r="A291" s="10" t="s">
+        <v>22</v>
       </c>
       <c r="B291" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C291" s="9">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="D291" s="4">
-        <v>32.164854642023002</v>
+        <v>61.609753215045302</v>
       </c>
       <c r="E291" s="6">
         <v>20</v>
       </c>
       <c r="F291" s="3">
         <f t="shared" si="6"/>
-        <v>25.731883713618402</v>
+        <v>49.287802572036242</v>
       </c>
       <c r="G291" s="1"/>
       <c r="H291" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="292" spans="1:8">
       <c r="A292" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B292" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C292" s="9">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="D292" s="4">
-        <v>34.249028517481499</v>
+        <v>33.456470827983601</v>
       </c>
       <c r="E292" s="6">
         <v>20</v>
       </c>
       <c r="F292" s="3">
         <f t="shared" si="6"/>
-        <v>27.399222813985197</v>
+        <v>26.765176662386882</v>
       </c>
       <c r="G292" s="1"/>
       <c r="H292" s="8" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
     </row>
     <row r="293" spans="1:8">
       <c r="A293" s="10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B293" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C293" s="9">
-        <v>73</v>
+        <v>139</v>
       </c>
       <c r="D293" s="4">
-        <v>56.364232531030197</v>
+        <v>64.038399660655003</v>
       </c>
       <c r="E293" s="6">
         <v>20</v>
       </c>
       <c r="F293" s="3">
         <f t="shared" si="6"/>
-        <v>45.09138602482416</v>
+        <v>51.230719728524001</v>
       </c>
       <c r="G293" s="1"/>
       <c r="H293" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="294" spans="1:8">
       <c r="A294" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B294" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C294" s="9">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="D294" s="4">
-        <v>29.681458688447002</v>
+        <v>88.3928023255814</v>
       </c>
       <c r="E294" s="6">
         <v>20</v>
       </c>
       <c r="F294" s="3">
         <f t="shared" si="6"/>
-        <v>23.7451669507576</v>
+        <v>70.714241860465123</v>
       </c>
       <c r="G294" s="1"/>
       <c r="H294" s="8" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
     </row>
     <row r="295" spans="1:8">
-      <c r="A295" s="10" t="s">
-        <v>24</v>
+      <c r="A295" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="B295" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C295" s="9">
-        <v>88</v>
+        <v>160</v>
       </c>
       <c r="D295" s="4">
-        <v>66.424341818395206</v>
+        <v>38.881013321004197</v>
       </c>
       <c r="E295" s="6">
         <v>20</v>
       </c>
       <c r="F295" s="3">
         <f t="shared" si="6"/>
-        <v>53.139473454716168</v>
+        <v>31.104810656803359</v>
       </c>
       <c r="G295" s="1"/>
       <c r="H295" s="8" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="296" spans="1:8">
-      <c r="A296" s="1" t="s">
-        <v>25</v>
+      <c r="A296" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="B296" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C296" s="9">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="D296" s="4">
-        <v>117.66158</v>
+        <v>52.267790172084403</v>
       </c>
       <c r="E296" s="6">
         <v>20</v>
       </c>
       <c r="F296" s="3">
         <f t="shared" si="6"/>
-        <v>94.129264000000006</v>
+        <v>41.814232137667524</v>
       </c>
       <c r="G296" s="1"/>
       <c r="H296" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="297" spans="1:8">
       <c r="A297" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B297" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C297" s="9">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="D297" s="4">
-        <v>32.019694007464103</v>
+        <v>126.401940695297</v>
       </c>
       <c r="E297" s="6">
         <v>20</v>
       </c>
       <c r="F297" s="3">
         <f t="shared" si="6"/>
-        <v>25.615755205971283</v>
+        <v>101.1215525562376</v>
       </c>
       <c r="G297" s="1"/>
       <c r="H297" s="8" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="298" spans="1:8">
-      <c r="A298" s="10" t="s">
-        <v>27</v>
+      <c r="A298" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="B298" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C298" s="9">
-        <v>77</v>
+        <v>168</v>
       </c>
       <c r="D298" s="4">
-        <v>45.581570352003197</v>
+        <v>34.397298925667798</v>
       </c>
       <c r="E298" s="6">
         <v>20</v>
       </c>
       <c r="F298" s="3">
         <f t="shared" si="6"/>
-        <v>36.465256281602556</v>
+        <v>27.517839140534239</v>
       </c>
       <c r="G298" s="1"/>
       <c r="H298" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="299" spans="1:8">
       <c r="A299" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B299" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C299" s="9">
-        <v>69</v>
+        <v>156</v>
       </c>
       <c r="D299" s="4">
-        <v>103.274454545455</v>
+        <v>31.755745670756699</v>
       </c>
       <c r="E299" s="6">
         <v>20</v>
       </c>
       <c r="F299" s="3">
         <f t="shared" si="6"/>
-        <v>82.619563636364006</v>
+        <v>25.404596536605361</v>
       </c>
       <c r="G299" s="1"/>
       <c r="H299" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="300" spans="1:8">
       <c r="A300" s="1" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="B300" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C300" s="9">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="D300" s="4">
-        <v>32.011510416666702</v>
+        <v>85.8098843963852</v>
       </c>
       <c r="E300" s="6">
         <v>20</v>
       </c>
       <c r="F300" s="3">
         <f t="shared" si="6"/>
-        <v>25.609208333333363</v>
+        <v>68.647907517108166</v>
       </c>
       <c r="G300" s="1"/>
       <c r="H300" s="8" t="s">
-        <v>98</v>
+        <v>138</v>
       </c>
     </row>
     <row r="301" spans="1:8">
-      <c r="A301" s="1" t="s">
-        <v>30</v>
+      <c r="A301" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="B301" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C301" s="9">
-        <v>85</v>
+        <v>141</v>
       </c>
       <c r="D301" s="4">
-        <v>41.469765200222</v>
+        <v>51.640695707107703</v>
       </c>
       <c r="E301" s="6">
         <v>20</v>
       </c>
       <c r="F301" s="3">
         <f t="shared" si="6"/>
-        <v>33.1758121601776</v>
+        <v>41.312556565686165</v>
       </c>
       <c r="G301" s="1"/>
       <c r="H301" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="302" spans="1:8">
       <c r="A302" s="1" t="s">
-        <v>137</v>
+        <v>32</v>
       </c>
       <c r="B302" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C302" s="9">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="D302" s="4">
-        <v>98.080272611832598</v>
+        <v>73.009943662951798</v>
       </c>
       <c r="E302" s="6">
         <v>20</v>
       </c>
       <c r="F302" s="3">
         <f t="shared" si="6"/>
-        <v>78.464218089466073</v>
+        <v>58.407954930361441</v>
       </c>
       <c r="G302" s="1"/>
       <c r="H302" s="8" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
     </row>
     <row r="303" spans="1:8">
-      <c r="A303" s="10" t="s">
-        <v>31</v>
+      <c r="A303" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="B303" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C303" s="9">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="D303" s="4">
-        <v>44.8543698230323</v>
+        <v>126.401940695297</v>
       </c>
       <c r="E303" s="6">
         <v>20</v>
       </c>
       <c r="F303" s="3">
         <f t="shared" si="6"/>
-        <v>35.883495858425839</v>
+        <v>101.1215525562376</v>
       </c>
       <c r="G303" s="1"/>
-      <c r="H303" s="8" t="s">
-        <v>100</v>
-      </c>
+      <c r="H303" s="8"/>
     </row>
     <row r="304" spans="1:8">
       <c r="A304" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B304" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C304" s="9">
-        <v>80</v>
+        <v>176</v>
       </c>
       <c r="D304" s="4">
-        <v>63.363835227272702</v>
+        <v>31.188293255131999</v>
       </c>
       <c r="E304" s="6">
         <v>20</v>
       </c>
       <c r="F304" s="3">
         <f t="shared" si="6"/>
-        <v>50.69106818181816</v>
+        <v>24.950634604105598</v>
       </c>
       <c r="G304" s="1"/>
       <c r="H304" s="8" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
     </row>
     <row r="305" spans="1:8">
       <c r="A305" s="1" t="s">
-        <v>141</v>
+        <v>34</v>
       </c>
       <c r="B305" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C305" s="9">
-        <v>16</v>
+        <v>166</v>
       </c>
       <c r="D305" s="4">
-        <v>103.274454545455</v>
+        <v>87.665935013964102</v>
       </c>
       <c r="E305" s="6">
         <v>20</v>
       </c>
       <c r="F305" s="3">
         <f t="shared" si="6"/>
-        <v>82.619563636364006</v>
+        <v>70.132748011171287</v>
       </c>
       <c r="G305" s="1"/>
-      <c r="H305" s="8"/>
+      <c r="H305" s="8" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="306" spans="1:8">
       <c r="A306" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B306" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C306" s="9">
-        <v>96</v>
+        <v>167</v>
       </c>
       <c r="D306" s="4">
-        <v>28.126445652173899</v>
+        <v>69.352811619718295</v>
       </c>
       <c r="E306" s="6">
         <v>20</v>
       </c>
       <c r="F306" s="3">
         <f t="shared" si="6"/>
-        <v>22.501156521739119</v>
+        <v>55.482249295774636</v>
       </c>
       <c r="G306" s="1"/>
       <c r="H306" s="8" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="307" spans="1:8">
       <c r="A307" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B307" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C307" s="9">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="D307" s="4">
-        <v>115.874940343171</v>
+        <v>36.535145325203302</v>
       </c>
       <c r="E307" s="6">
         <v>20</v>
       </c>
       <c r="F307" s="3">
         <f t="shared" si="6"/>
-        <v>92.699952274536798</v>
+        <v>29.228116260162643</v>
       </c>
       <c r="G307" s="1"/>
       <c r="H307" s="8" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="308" spans="1:8">
-      <c r="A308" s="1" t="s">
-        <v>35</v>
+      <c r="A308" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="B308" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C308" s="9">
-        <v>87</v>
+        <v>163</v>
       </c>
       <c r="D308" s="4">
-        <v>64.704009900990101</v>
+        <v>65.116759665642803</v>
       </c>
       <c r="E308" s="6">
         <v>20</v>
       </c>
       <c r="F308" s="3">
         <f t="shared" si="6"/>
-        <v>51.763207920792084</v>
+        <v>52.093407732514244</v>
       </c>
       <c r="G308" s="1"/>
       <c r="H308" s="8" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
     </row>
     <row r="309" spans="1:8">
       <c r="A309" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B309" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C309" s="9">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D309" s="4">
-        <v>31.229027243589702</v>
+        <v>72.692134156806901</v>
       </c>
       <c r="E309" s="6">
         <v>20</v>
       </c>
       <c r="F309" s="3">
         <f t="shared" si="6"/>
-        <v>24.98322179487176</v>
+        <v>58.153707325445524</v>
       </c>
       <c r="G309" s="1"/>
       <c r="H309" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="310" spans="1:8">
-      <c r="A310" s="10" t="s">
-        <v>37</v>
+      <c r="A310" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="B310" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C310" s="9">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="D310" s="4">
-        <v>66.972437992236706</v>
+        <v>118.356012267064</v>
       </c>
       <c r="E310" s="6">
         <v>20</v>
       </c>
       <c r="F310" s="3">
         <f t="shared" si="6"/>
-        <v>53.577950393789365</v>
+        <v>94.684809813651199</v>
       </c>
       <c r="G310" s="1"/>
       <c r="H310" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="311" spans="1:8">
       <c r="A311" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B311" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C311" s="9">
-        <v>88</v>
+        <v>156</v>
       </c>
       <c r="D311" s="4">
-        <v>63.363835227272702</v>
+        <v>43.0334627677342</v>
       </c>
       <c r="E311" s="6">
         <v>20</v>
       </c>
       <c r="F311" s="3">
         <f t="shared" si="6"/>
-        <v>50.69106818181816</v>
+        <v>34.426770214187357</v>
       </c>
       <c r="G311" s="1"/>
       <c r="H311" s="8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="312" spans="1:8">
       <c r="A312" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B312" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C312" s="9">
-        <v>62</v>
+        <v>154</v>
       </c>
       <c r="D312" s="4">
-        <v>93.173415097909398</v>
+        <v>29.255522727272702</v>
       </c>
       <c r="E312" s="6">
         <v>20</v>
       </c>
       <c r="F312" s="3">
         <f t="shared" si="6"/>
-        <v>74.538732078327513</v>
+        <v>23.404418181818162</v>
       </c>
       <c r="G312" s="1"/>
       <c r="H312" s="8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="313" spans="1:8">
       <c r="A313" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B313" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C313" s="9">
-        <v>84</v>
+        <v>152</v>
       </c>
       <c r="D313" s="4">
-        <v>69.129963316404897</v>
+        <v>39.122489596083199</v>
       </c>
       <c r="E313" s="6">
         <v>20</v>
       </c>
       <c r="F313" s="3">
         <f t="shared" si="6"/>
-        <v>55.303970653123919</v>
+        <v>31.297991676866559</v>
       </c>
       <c r="G313" s="1"/>
       <c r="H313" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="314" spans="1:8">
       <c r="A314" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B314" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C314" s="9">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="D314" s="4">
-        <v>27.2976363636364</v>
+        <v>44.091314393939399</v>
       </c>
       <c r="E314" s="6">
         <v>20</v>
       </c>
       <c r="F314" s="3">
         <f t="shared" si="6"/>
-        <v>21.838109090909121</v>
+        <v>35.273051515151522</v>
       </c>
       <c r="G314" s="1"/>
       <c r="H314" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="315" spans="1:8">
       <c r="A315" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B315" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C315" s="9">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="D315" s="4">
-        <v>38.761173333333304</v>
+        <v>138.055726689957</v>
       </c>
       <c r="E315" s="6">
         <v>20</v>
       </c>
       <c r="F315" s="3">
         <f t="shared" si="6"/>
-        <v>31.008938666666644</v>
+        <v>110.4445813519656</v>
       </c>
       <c r="G315" s="1"/>
       <c r="H315" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="316" spans="1:8">
       <c r="A316" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B316" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C316" s="9">
-        <v>72</v>
+        <v>116</v>
       </c>
       <c r="D316" s="4">
-        <v>36.366624999999999</v>
+        <v>33.228430586413999</v>
       </c>
       <c r="E316" s="6">
         <v>20</v>
       </c>
       <c r="F316" s="3">
         <f t="shared" si="6"/>
-        <v>29.093299999999999</v>
+        <v>26.5827444691312</v>
       </c>
       <c r="G316" s="1"/>
       <c r="H316" s="8" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
     </row>
     <row r="317" spans="1:8">
       <c r="A317" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B317" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C317" s="9"/>
-      <c r="D317" s="4"/>
+        <v>45991</v>
+      </c>
+      <c r="C317" s="9">
+        <v>176</v>
+      </c>
+      <c r="D317" s="4">
+        <v>42.893889259977797</v>
+      </c>
       <c r="E317" s="6">
         <v>20</v>
       </c>
       <c r="F317" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>34.315111407982236</v>
       </c>
       <c r="G317" s="1"/>
       <c r="H317" s="8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="318" spans="1:8">
-      <c r="A318" s="1" t="s">
-        <v>45</v>
+      <c r="A318" s="10" t="s">
+        <v>47</v>
       </c>
       <c r="B318" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C318" s="9">
-        <v>68</v>
+        <v>176</v>
       </c>
       <c r="D318" s="4">
-        <v>30.1475120048019</v>
+        <v>69.352811619718295</v>
       </c>
       <c r="E318" s="6">
         <v>20</v>
       </c>
       <c r="F318" s="3">
         <f t="shared" si="6"/>
-        <v>24.118009603841521</v>
+        <v>55.482249295774636</v>
       </c>
       <c r="G318" s="1"/>
       <c r="H318" s="8" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
     </row>
     <row r="319" spans="1:8">
-      <c r="A319" s="1" t="s">
-        <v>46</v>
+      <c r="A319" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="B319" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C319" s="9">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="D319" s="4">
-        <v>49.737972826087002</v>
+        <v>69.352811619718295</v>
       </c>
       <c r="E319" s="6">
         <v>20</v>
       </c>
       <c r="F319" s="3">
         <f t="shared" si="6"/>
-        <v>39.790378260869602</v>
+        <v>55.482249295774636</v>
       </c>
       <c r="G319" s="1"/>
       <c r="H319" s="8" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="320" spans="1:8">
-      <c r="A320" s="10" t="s">
-        <v>47</v>
+      <c r="A320" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="B320" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C320" s="9">
-        <v>96</v>
+        <v>184</v>
       </c>
       <c r="D320" s="4">
-        <v>64.704009900990101</v>
+        <v>35.764634634387299</v>
       </c>
       <c r="E320" s="6">
         <v>20</v>
       </c>
       <c r="F320" s="3">
         <f t="shared" si="6"/>
-        <v>51.763207920792084</v>
+        <v>28.61170770750984</v>
       </c>
       <c r="G320" s="1"/>
       <c r="H320" s="8" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="321" spans="1:8">
-      <c r="A321" s="10" t="s">
-        <v>48</v>
+      <c r="A321" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="B321" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C321" s="9">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D321" s="4">
-        <v>64.704009900990101</v>
+        <v>53.564347826086902</v>
       </c>
       <c r="E321" s="6">
         <v>20</v>
       </c>
       <c r="F321" s="3">
         <f t="shared" si="6"/>
-        <v>51.763207920792084</v>
+        <v>42.85147826086952</v>
       </c>
       <c r="G321" s="1"/>
       <c r="H321" s="8" t="s">
-        <v>72</v>
+        <v>124</v>
       </c>
     </row>
     <row r="322" spans="1:8">
       <c r="A322" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B322" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C322" s="9">
-        <v>112</v>
+        <v>176</v>
       </c>
       <c r="D322" s="4">
-        <v>29.926879464285701</v>
+        <v>35.448980113636303</v>
       </c>
       <c r="E322" s="6">
         <v>20</v>
       </c>
       <c r="F322" s="3">
         <f t="shared" si="6"/>
-        <v>23.941503571428562</v>
+        <v>28.359184090909043</v>
       </c>
       <c r="G322" s="1"/>
       <c r="H322" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="323" spans="1:8">
       <c r="A323" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B323" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C323" s="9">
-        <v>96</v>
+        <v>184</v>
       </c>
       <c r="D323" s="4">
-        <v>48.371413043478199</v>
+        <v>47.900705877298499</v>
       </c>
       <c r="E323" s="6">
         <v>20</v>
       </c>
       <c r="F323" s="3">
         <f t="shared" si="6"/>
-        <v>38.697130434782558</v>
+        <v>38.320564701838798</v>
       </c>
       <c r="G323" s="1"/>
       <c r="H323" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="324" spans="1:8">
       <c r="A324" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B324" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C324" s="9">
-        <v>104</v>
+        <v>168</v>
       </c>
       <c r="D324" s="4">
-        <v>29.447552884615401</v>
+        <v>35.043873962999797</v>
       </c>
       <c r="E324" s="6">
         <v>20</v>
       </c>
       <c r="F324" s="3">
         <f t="shared" si="6"/>
-        <v>23.558042307692322</v>
+        <v>28.035099170399839</v>
       </c>
       <c r="G324" s="1"/>
       <c r="H324" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
     </row>
     <row r="325" spans="1:8">
       <c r="A325" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B325" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C325" s="9">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="D325" s="4">
-        <v>46.492445652173899</v>
+        <v>34.037200887328602</v>
       </c>
       <c r="E325" s="6">
         <v>20</v>
       </c>
       <c r="F325" s="3">
         <f t="shared" si="6"/>
-        <v>37.193956521739118</v>
+        <v>27.22976070986288</v>
       </c>
       <c r="G325" s="1"/>
       <c r="H325" s="8" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
     </row>
     <row r="326" spans="1:8">
       <c r="A326" s="1" t="s">
-        <v>53</v>
+        <v>152</v>
       </c>
       <c r="B326" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C326" s="9">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="D326" s="4">
-        <v>32.176956559829101</v>
+        <v>126.401940695297</v>
       </c>
       <c r="E326" s="6">
         <v>20</v>
       </c>
       <c r="F326" s="3">
         <f t="shared" si="6"/>
-        <v>25.741565247863281</v>
+        <v>101.1215525562376</v>
       </c>
       <c r="G326" s="1"/>
-      <c r="H326" s="8" t="s">
-        <v>115</v>
-      </c>
+      <c r="H326" s="8"/>
     </row>
     <row r="327" spans="1:8">
       <c r="A327" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B327" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C327" s="9">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="D327" s="4">
-        <v>31.346785496470499</v>
+        <v>34.774626321423803</v>
       </c>
       <c r="E327" s="6">
         <v>20</v>
       </c>
       <c r="F327" s="3">
         <f t="shared" si="6"/>
-        <v>25.077428397176398</v>
+        <v>27.819701057139042</v>
       </c>
       <c r="G327" s="1"/>
       <c r="H327" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="328" spans="1:8">
       <c r="A328" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B328" s="7">
+        <v>45991</v>
+      </c>
+      <c r="C328" s="9">
         <v>152</v>
       </c>
-      <c r="B328" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C328" s="9">
-        <v>13</v>
-      </c>
       <c r="D328" s="4">
-        <v>103.274454545455</v>
+        <v>32.023106772613403</v>
       </c>
       <c r="E328" s="6">
         <v>20</v>
       </c>
       <c r="F328" s="3">
         <f t="shared" si="6"/>
-        <v>82.619563636364006</v>
+        <v>25.618485418090721</v>
       </c>
       <c r="G328" s="1"/>
-      <c r="H328" s="8"/>
+      <c r="H328" s="8" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="329" spans="1:8">
       <c r="A329" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B329" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C329" s="9">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="D329" s="4">
-        <v>32.350611342992899</v>
+        <v>34.662226704545397</v>
       </c>
       <c r="E329" s="6">
         <v>20</v>
       </c>
       <c r="F329" s="3">
         <f t="shared" si="6"/>
-        <v>25.880489074394319</v>
+        <v>27.729781363636317</v>
       </c>
       <c r="G329" s="1"/>
       <c r="H329" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="330" spans="1:8">
       <c r="A330" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B330" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C330" s="9">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="D330" s="4">
-        <v>30.421940789473702</v>
+        <v>41.266697646467001</v>
       </c>
       <c r="E330" s="6">
         <v>20</v>
       </c>
       <c r="F330" s="3">
         <f t="shared" si="6"/>
-        <v>24.337552631578962</v>
+        <v>33.013358117173603</v>
       </c>
       <c r="G330" s="1"/>
       <c r="H330" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="331" spans="1:8">
       <c r="A331" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B331" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C331" s="9">
-        <v>88</v>
+        <v>128</v>
       </c>
       <c r="D331" s="4">
-        <v>32.660236742424303</v>
+        <v>32.388312499999998</v>
       </c>
       <c r="E331" s="6">
         <v>20</v>
       </c>
       <c r="F331" s="3">
         <f t="shared" si="6"/>
-        <v>26.128189393939444</v>
+        <v>25.910649999999997</v>
       </c>
       <c r="G331" s="1"/>
       <c r="H331" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="332" spans="1:8">
       <c r="A332" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B332" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C332" s="9">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="D332" s="4">
-        <v>40.3757801390529</v>
+        <v>44.936636595744702</v>
       </c>
       <c r="E332" s="6">
         <v>20</v>
       </c>
       <c r="F332" s="3">
         <f t="shared" si="6"/>
-        <v>32.300624111242321</v>
+        <v>35.949309276595763</v>
       </c>
       <c r="G332" s="1"/>
       <c r="H332" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="333" spans="1:8">
       <c r="A333" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B333" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C333" s="9">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="D333" s="4">
-        <v>34.434678571428599</v>
+        <v>46.078225000000003</v>
       </c>
       <c r="E333" s="6">
         <v>20</v>
       </c>
       <c r="F333" s="3">
         <f t="shared" si="6"/>
-        <v>27.547742857142879</v>
+        <v>36.862580000000001</v>
       </c>
       <c r="G333" s="1"/>
       <c r="H333" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="334" spans="1:8">
       <c r="A334" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B334" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C334" s="9">
-        <v>48</v>
+        <v>168</v>
       </c>
       <c r="D334" s="4">
-        <v>38.463169312169299</v>
+        <v>38.524439547383999</v>
       </c>
       <c r="E334" s="6">
         <v>20</v>
       </c>
       <c r="F334" s="3">
         <f t="shared" si="6"/>
-        <v>30.770535449735441</v>
+        <v>30.8195516379072</v>
       </c>
       <c r="G334" s="1"/>
       <c r="H334" s="8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="335" spans="1:8">
       <c r="A335" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B335" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C335" s="9">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="D335" s="4">
-        <v>40.651797619047599</v>
+        <v>55.400851106519198</v>
       </c>
       <c r="E335" s="6">
         <v>20</v>
       </c>
       <c r="F335" s="3">
         <f t="shared" si="6"/>
-        <v>32.521438095238082</v>
+        <v>44.32068088521536</v>
       </c>
       <c r="G335" s="1"/>
       <c r="H335" s="8" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="336" spans="1:8">
       <c r="A336" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B336" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C336" s="9">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="D336" s="4">
-        <v>41.4668669481606</v>
+        <v>122.259504428672</v>
       </c>
       <c r="E336" s="6">
         <v>20</v>
       </c>
       <c r="F336" s="3">
         <f t="shared" si="6"/>
-        <v>33.173493558528477</v>
+        <v>97.807603542937599</v>
       </c>
       <c r="G336" s="1"/>
       <c r="H336" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="337" spans="1:8">
       <c r="A337" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B337" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C337" s="9">
-        <v>64</v>
+        <v>176</v>
       </c>
       <c r="D337" s="4">
-        <v>56.425414381099102</v>
+        <v>42.763601458579302</v>
       </c>
       <c r="E337" s="6">
         <v>20</v>
       </c>
       <c r="F337" s="3">
-        <f t="shared" si="6"/>
-        <v>45.140331504879285</v>
+        <f t="shared" ref="F337:F342" si="7">D337-(D337*E337)/100</f>
+        <v>34.210881166863444</v>
       </c>
       <c r="G337" s="1"/>
       <c r="H337" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="338" spans="1:8">
-      <c r="A338" s="1" t="s">
-        <v>64</v>
+      <c r="A338" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="B338" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C338" s="9">
-        <v>21</v>
+        <v>144</v>
       </c>
       <c r="D338" s="4">
-        <v>107.8525579528</v>
+        <v>71.2247082005441</v>
       </c>
       <c r="E338" s="6">
         <v>20</v>
       </c>
       <c r="F338" s="3">
-        <f t="shared" si="6"/>
-        <v>86.282046362239996</v>
+        <f t="shared" si="7"/>
+        <v>56.97976656043528</v>
       </c>
       <c r="G338" s="1"/>
-      <c r="H338" s="8" t="s">
-        <v>130</v>
-      </c>
+      <c r="H338" s="8"/>
     </row>
     <row r="339" spans="1:8">
       <c r="A339" s="1" t="s">
-        <v>65</v>
+        <v>133</v>
       </c>
       <c r="B339" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C339" s="9">
-        <v>104</v>
+        <v>154</v>
       </c>
       <c r="D339" s="4">
-        <v>38.006612446581201</v>
+        <v>29.255522727272702</v>
       </c>
       <c r="E339" s="6">
         <v>20</v>
       </c>
       <c r="F339" s="3">
-        <f t="shared" ref="F339:F344" si="7">D339-(D339*E339)/100</f>
-        <v>30.405289957264962</v>
+        <f t="shared" si="7"/>
+        <v>23.404418181818162</v>
       </c>
       <c r="G339" s="1"/>
-      <c r="H339" s="8" t="s">
-        <v>131</v>
-      </c>
+      <c r="H339" s="8"/>
     </row>
     <row r="340" spans="1:8">
-      <c r="A340" s="10" t="s">
-        <v>134</v>
+      <c r="A340" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="B340" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C340" s="9">
-        <v>80</v>
-      </c>
-      <c r="D340" s="4">
-        <v>89.243906249999995</v>
-      </c>
+        <v>45991</v>
+      </c>
+      <c r="C340" s="9"/>
+      <c r="D340" s="4"/>
       <c r="E340" s="6">
         <v>20</v>
       </c>
       <c r="F340" s="3">
         <f t="shared" si="7"/>
-        <v>71.395124999999993</v>
+        <v>0</v>
       </c>
       <c r="G340" s="1"/>
       <c r="H340" s="8"/>
     </row>
     <row r="341" spans="1:8">
       <c r="A341" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B341" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C341" s="9">
-        <v>88</v>
+        <v>184</v>
       </c>
       <c r="D341" s="4">
-        <v>27.2976363636364</v>
+        <v>43.976640382483303</v>
       </c>
       <c r="E341" s="6">
         <v>20</v>
       </c>
       <c r="F341" s="3">
         <f t="shared" si="7"/>
-        <v>21.838109090909121</v>
+        <v>35.181312305986644</v>
       </c>
       <c r="G341" s="1"/>
       <c r="H341" s="8"/>
     </row>
     <row r="342" spans="1:8">
       <c r="A342" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B342" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C342" s="9"/>
-      <c r="D342" s="4"/>
+        <v>45991</v>
+      </c>
+      <c r="C342" s="9">
+        <v>24</v>
+      </c>
+      <c r="D342" s="4">
+        <v>178.00537837991399</v>
+      </c>
       <c r="E342" s="6">
         <v>20</v>
       </c>
       <c r="F342" s="3">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>142.40430270393119</v>
       </c>
       <c r="G342" s="1"/>
       <c r="H342" s="8"/>
     </row>
     <row r="343" spans="1:8">
       <c r="A343" s="1" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="B343" s="7">
-        <v>45979</v>
+        <v>45991</v>
       </c>
       <c r="C343" s="9">
-        <v>104</v>
+        <v>37</v>
       </c>
       <c r="D343" s="4">
-        <v>50.264938719342197</v>
+        <v>126.401940695297</v>
       </c>
       <c r="E343" s="6">
         <v>20</v>
       </c>
       <c r="F343" s="3">
-        <f t="shared" si="7"/>
-        <v>40.211950975473755</v>
+        <f t="shared" ref="F343" si="8">D343-(D343*E343)/100</f>
+        <v>101.1215525562376</v>
       </c>
       <c r="G343" s="1"/>
       <c r="H343" s="8"/>
-    </row>
-    <row r="344" spans="1:8">
-      <c r="A344" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B344" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C344" s="9"/>
-      <c r="D344" s="4"/>
-      <c r="E344" s="6">
-        <v>20</v>
-      </c>
-      <c r="F344" s="3">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="G344" s="1"/>
-      <c r="H344" s="8"/>
-    </row>
-    <row r="345" spans="1:8">
-      <c r="A345" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B345" s="7">
-        <v>45979</v>
-      </c>
-      <c r="C345" s="9">
-        <v>37</v>
-      </c>
-      <c r="D345" s="4">
-        <v>103.274454545455</v>
-      </c>
-      <c r="E345" s="6">
-        <v>20</v>
-      </c>
-      <c r="F345" s="3">
-        <f t="shared" ref="F345" si="8">D345-(D345*E345)/100</f>
-        <v>82.619563636364006</v>
-      </c>
-      <c r="G345" s="1"/>
-      <c r="H345" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G272"/>
@@ -9697,7 +9665,7 @@
     <hyperlink ref="H283" r:id="rId265"/>
     <hyperlink ref="H284" r:id="rId266"/>
     <hyperlink ref="H285" r:id="rId267"/>
-    <hyperlink ref="H286" r:id="rId268"/>
+    <hyperlink ref="H287" r:id="rId268"/>
     <hyperlink ref="H288" r:id="rId269"/>
     <hyperlink ref="H289" r:id="rId270"/>
     <hyperlink ref="H290" r:id="rId271"/>
@@ -9710,10 +9678,10 @@
     <hyperlink ref="H297" r:id="rId278"/>
     <hyperlink ref="H298" r:id="rId279"/>
     <hyperlink ref="H299" r:id="rId280"/>
-    <hyperlink ref="H300" r:id="rId281"/>
-    <hyperlink ref="H301" r:id="rId282"/>
-    <hyperlink ref="H303" r:id="rId283"/>
-    <hyperlink ref="H304" r:id="rId284"/>
+    <hyperlink ref="H301" r:id="rId281"/>
+    <hyperlink ref="H302" r:id="rId282"/>
+    <hyperlink ref="H304" r:id="rId283"/>
+    <hyperlink ref="H305" r:id="rId284"/>
     <hyperlink ref="H306" r:id="rId285"/>
     <hyperlink ref="H307" r:id="rId286"/>
     <hyperlink ref="H308" r:id="rId287"/>
@@ -9734,8 +9702,8 @@
     <hyperlink ref="H323" r:id="rId302"/>
     <hyperlink ref="H324" r:id="rId303"/>
     <hyperlink ref="H325" r:id="rId304"/>
-    <hyperlink ref="H326" r:id="rId305"/>
-    <hyperlink ref="H327" r:id="rId306"/>
+    <hyperlink ref="H327" r:id="rId305"/>
+    <hyperlink ref="H328" r:id="rId306"/>
     <hyperlink ref="H329" r:id="rId307"/>
     <hyperlink ref="H330" r:id="rId308"/>
     <hyperlink ref="H331" r:id="rId309"/>
@@ -9745,9 +9713,7 @@
     <hyperlink ref="H335" r:id="rId313"/>
     <hyperlink ref="H336" r:id="rId314"/>
     <hyperlink ref="H337" r:id="rId315"/>
-    <hyperlink ref="H338" r:id="rId316"/>
-    <hyperlink ref="H339" r:id="rId317"/>
-    <hyperlink ref="H302" r:id="rId318" display="mailto:cyborg.3@hotmail.it"/>
+    <hyperlink ref="H300" r:id="rId316" display="mailto:cyborg.3@hotmail.it"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>